<commit_message>
Fix level order in cell subtype colors
</commit_message>
<xml_diff>
--- a/processed-data/04_snRNA-seq/27.5_sn_neuron_check/ERC_neuron_subcluster_details_annotated.xlsx
+++ b/processed-data/04_snRNA-seq/27.5_sn_neuron_check/ERC_neuron_subcluster_details_annotated.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lieberinstitute-my.sharepoint.com/personal/louise_huuki_libd_org/Documents/LIBD_code/LFF_spatial_ERC/processed-data/04_snRNA-seq/27.5_sn_neuron_check/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{29615A01-63BA-C041-9294-ED5917662BBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CE8334E8-8E38-7446-ABA9-F128B376F6C2}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="13_ncr:1_{29615A01-63BA-C041-9294-ED5917662BBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E513D9DC-E5AD-DD4E-8727-42155D97246E}"/>
   <bookViews>
-    <workbookView xWindow="60" yWindow="660" windowWidth="30240" windowHeight="17580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="206">
   <si>
     <t>cell_type_anno</t>
   </si>
@@ -502,21 +502,6 @@
     <t>CGE-derived VIP+ disinhibitory interneuron population. VIP and CALB2 (calretinin, classically co-expressed with VIP in cortical interneurons) are both confirmed as top global markers, alongside SP8 and HTR3A -- the latter shared with Inhib.Htr3a, consistent with both populations being the VIP-positive and VIP-negative halves of the same 5HT3aR+ interneuron class. Sestan resolves four VIP sub-populations collapsed into this one cluster -- worth revisiting at higher resolution if finer VIP heterogeneity matters for the study.</t>
   </si>
   <si>
-    <t>clean L5 signal conflicts with RELN  label - high RELN expression - not as high as ExcitL5.2</t>
-  </si>
-  <si>
-    <t>low expression of ETV1</t>
-  </si>
-  <si>
-    <t>high expression of BCL11B, highest expression of RELN</t>
-  </si>
-  <si>
-    <t>Excit.L5_RELN</t>
-  </si>
-  <si>
-    <t>Excit.L5_RORB</t>
-  </si>
-  <si>
     <t>Excit.L2_5.RELN</t>
   </si>
   <si>
@@ -619,16 +604,47 @@
     <t>CALB2, ADRA1B, CCNG2, PROX1, DLX1</t>
   </si>
   <si>
-    <t xml:space="preserve">passed strict QC filtering </t>
-  </si>
-  <si>
-    <t>Excit.L2_5.diffuse</t>
-  </si>
-  <si>
     <t xml:space="preserve">RELN+ population (also CUX2+, ADARB2+, BMPR1B+), part of the classic Layer II stellate/fan-cell, DG-projecting (perforant path) lineage described by Nilssen et al. 2019 and Witter et al. 2017. Spatial registration in both Visium (vL5a) and Xenium (xL5, 72%) places it deeper than that molecular identity alone would predict; it is also the closest global transcriptomic neighbor of Excit.L5.2 (their top marker genes reciprocally rank each other as nearest competitor), consistent with their shared position as sister branches in the dendrogram. </t>
   </si>
   <si>
     <t>SR ERC splits, but xenium and Sestan lean L2</t>
+  </si>
+  <si>
+    <t>clean L5 signal conflicts with RELN  label - high RELN expression - not as high as ExcitL5.2
+spatail match</t>
+  </si>
+  <si>
+    <t>low expression of ETV1
+multiple spatail reg, L5 strongest match</t>
+  </si>
+  <si>
+    <t>L5_6 confirmed w/ spatial</t>
+  </si>
+  <si>
+    <t>L6 confirmed w/ spatial</t>
+  </si>
+  <si>
+    <t>worst QC but passed strict QC filtering
+multiple layer matches</t>
+  </si>
+  <si>
+    <t>high expression of BCL11B, highest expression of RELN
+Xenium shows L2_5 split - only register to L5a</t>
+  </si>
+  <si>
+    <t>Excit.L2_5.mix</t>
+  </si>
+  <si>
+    <t>Excit.L5.RELN</t>
+  </si>
+  <si>
+    <t>Excit.L5.RORB</t>
+  </si>
+  <si>
+    <t>Excit.L5_6.NP</t>
+  </si>
+  <si>
+    <t>Excit.L6.CT</t>
   </si>
 </sst>
 </file>
@@ -683,7 +699,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -693,6 +709,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1022,7 +1041,7 @@
     <col min="10" max="10" width="8.83203125" style="1"/>
     <col min="12" max="12" width="12.33203125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="19.1640625" style="3" customWidth="1"/>
-    <col min="16" max="16" width="19.83203125" customWidth="1"/>
+    <col min="16" max="16" width="19.83203125" style="3" customWidth="1"/>
     <col min="18" max="18" width="15.5" customWidth="1"/>
     <col min="19" max="19" width="15.33203125" customWidth="1"/>
     <col min="20" max="20" width="93.5" style="4" customWidth="1"/>
@@ -1078,7 +1097,7 @@
       <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="3" t="s">
         <v>15</v>
       </c>
       <c r="Q1" t="s">
@@ -1155,7 +1174,7 @@
       <c r="O2" t="s">
         <v>89</v>
       </c>
-      <c r="P2" s="4" t="s">
+      <c r="P2" s="5" t="s">
         <v>101</v>
       </c>
       <c r="Q2" t="s">
@@ -1171,7 +1190,7 @@
         <v>146</v>
       </c>
       <c r="U2" s="4" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="V2" t="s">
         <v>25</v>
@@ -1180,10 +1199,10 @@
         <v>0</v>
       </c>
       <c r="X2" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="Y2" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
     </row>
     <row r="3" spans="1:25" ht="128" x14ac:dyDescent="0.2">
@@ -1232,7 +1251,7 @@
       <c r="O3" t="s">
         <v>89</v>
       </c>
-      <c r="P3" s="4" t="s">
+      <c r="P3" s="5" t="s">
         <v>102</v>
       </c>
       <c r="Q3" t="s">
@@ -1247,25 +1266,25 @@
       <c r="T3" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="U3" t="s">
-        <v>198</v>
+      <c r="U3" s="4" t="s">
+        <v>199</v>
       </c>
       <c r="V3" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="W3" t="b">
         <v>1</v>
       </c>
       <c r="X3" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="Y3" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
     </row>
-    <row r="4" spans="1:25" ht="80" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:25" ht="112" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B4" t="s">
         <v>39</v>
@@ -1274,25 +1293,25 @@
         <v>40</v>
       </c>
       <c r="D4" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E4">
-        <v>609</v>
+        <v>241</v>
       </c>
       <c r="F4" s="2">
-        <v>4.8455240565549E-3</v>
+        <v>1.9175226562064E-3</v>
       </c>
       <c r="G4">
-        <v>61717</v>
+        <v>63691</v>
       </c>
       <c r="H4">
-        <v>9080</v>
+        <v>9154</v>
       </c>
       <c r="I4" s="1">
-        <v>3.2713949227950803E-2</v>
+        <v>3.69902018976834E-2</v>
       </c>
       <c r="J4" s="1">
-        <v>1.2973302509634999E-3</v>
+        <v>5.1066987216472001E-3</v>
       </c>
       <c r="K4" t="b">
         <v>1</v>
@@ -1301,48 +1320,48 @@
         <v>58</v>
       </c>
       <c r="M4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="O4" t="s">
-        <v>90</v>
-      </c>
-      <c r="P4" s="4" t="s">
-        <v>103</v>
+        <v>92</v>
+      </c>
+      <c r="P4" s="5" t="s">
+        <v>105</v>
       </c>
       <c r="Q4" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="R4" s="4" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="S4" s="4" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="T4" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="U4" s="4" t="s">
         <v>200</v>
       </c>
-      <c r="U4" t="s">
+      <c r="V4" t="s">
         <v>159</v>
       </c>
-      <c r="V4" t="s">
-        <v>162</v>
-      </c>
       <c r="W4" t="b">
         <v>1</v>
       </c>
       <c r="X4" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="Y4" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
     </row>
-    <row r="5" spans="1:25" ht="64" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:25" ht="80" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B5" t="s">
         <v>39</v>
@@ -1351,75 +1370,75 @@
         <v>40</v>
       </c>
       <c r="D5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E5">
-        <v>2235</v>
+        <v>609</v>
       </c>
       <c r="F5" s="2">
-        <v>1.7782834591790499E-2</v>
+        <v>4.8455240565549E-3</v>
       </c>
       <c r="G5">
-        <v>57008</v>
+        <v>61717</v>
       </c>
       <c r="H5">
-        <v>8821</v>
+        <v>9080</v>
       </c>
       <c r="I5" s="1">
-        <v>0.11163545948140299</v>
+        <v>3.2713949227950803E-2</v>
       </c>
       <c r="J5" s="1">
-        <v>2.3670920636503999E-3</v>
+        <v>1.2973302509634999E-3</v>
       </c>
       <c r="K5" t="b">
         <v>1</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="N5" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="O5" t="s">
-        <v>91</v>
-      </c>
-      <c r="P5" s="4" t="s">
-        <v>104</v>
+        <v>90</v>
+      </c>
+      <c r="P5" s="5" t="s">
+        <v>103</v>
       </c>
       <c r="Q5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="R5" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="S5" s="4" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="T5" s="4" t="s">
-        <v>148</v>
-      </c>
-      <c r="U5" t="s">
-        <v>160</v>
+        <v>193</v>
+      </c>
+      <c r="U5" s="4" t="s">
+        <v>195</v>
       </c>
       <c r="V5" t="s">
-        <v>163</v>
+        <v>202</v>
       </c>
       <c r="W5" t="b">
         <v>1</v>
       </c>
       <c r="X5" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="Y5" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
     </row>
-    <row r="6" spans="1:25" ht="112" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:25" ht="64" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B6" t="s">
         <v>39</v>
@@ -1428,70 +1447,70 @@
         <v>40</v>
       </c>
       <c r="D6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E6">
-        <v>241</v>
+        <v>2235</v>
       </c>
       <c r="F6" s="2">
-        <v>1.9175226562064E-3</v>
+        <v>1.7782834591790499E-2</v>
       </c>
       <c r="G6">
-        <v>63691</v>
+        <v>57008</v>
       </c>
       <c r="H6">
-        <v>9154</v>
+        <v>8821</v>
       </c>
       <c r="I6" s="1">
-        <v>3.69902018976834E-2</v>
+        <v>0.11163545948140299</v>
       </c>
       <c r="J6" s="1">
-        <v>5.1066987216472001E-3</v>
+        <v>2.3670920636503999E-3</v>
       </c>
       <c r="K6" t="b">
         <v>1</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="M6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="N6" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O6" t="s">
-        <v>92</v>
-      </c>
-      <c r="P6" s="4" t="s">
-        <v>105</v>
+        <v>91</v>
+      </c>
+      <c r="P6" s="5" t="s">
+        <v>104</v>
       </c>
       <c r="Q6" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="R6" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="S6" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="T6" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="U6" t="s">
-        <v>161</v>
+        <v>148</v>
+      </c>
+      <c r="U6" s="4" t="s">
+        <v>196</v>
       </c>
       <c r="V6" t="s">
-        <v>164</v>
+        <v>203</v>
       </c>
       <c r="W6" t="b">
         <v>1</v>
       </c>
       <c r="X6" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="Y6" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
     </row>
     <row r="7" spans="1:25" ht="112" x14ac:dyDescent="0.2">
@@ -1540,7 +1559,7 @@
       <c r="O7" t="s">
         <v>93</v>
       </c>
-      <c r="P7" s="4" t="s">
+      <c r="P7" s="5" t="s">
         <v>106</v>
       </c>
       <c r="R7" s="4" t="s">
@@ -1552,17 +1571,20 @@
       <c r="T7" s="4" t="s">
         <v>150</v>
       </c>
+      <c r="U7" s="4" t="s">
+        <v>197</v>
+      </c>
       <c r="V7" t="s">
-        <v>30</v>
+        <v>204</v>
       </c>
       <c r="W7" t="b">
         <v>0</v>
       </c>
       <c r="X7" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="Y7" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
     </row>
     <row r="8" spans="1:25" ht="80" x14ac:dyDescent="0.2">
@@ -1611,7 +1633,7 @@
       <c r="O8" t="s">
         <v>94</v>
       </c>
-      <c r="P8" s="4" t="s">
+      <c r="P8" s="5" t="s">
         <v>107</v>
       </c>
       <c r="R8" s="4" t="s">
@@ -1623,17 +1645,20 @@
       <c r="T8" s="4" t="s">
         <v>151</v>
       </c>
+      <c r="U8" t="s">
+        <v>198</v>
+      </c>
       <c r="V8" t="s">
-        <v>31</v>
+        <v>205</v>
       </c>
       <c r="W8" t="b">
         <v>0</v>
       </c>
       <c r="X8" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="Y8" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
     </row>
     <row r="9" spans="1:25" ht="80" x14ac:dyDescent="0.2">
@@ -1682,7 +1707,7 @@
       <c r="O9" t="s">
         <v>69</v>
       </c>
-      <c r="P9" s="4" t="s">
+      <c r="P9" s="5" t="s">
         <v>107</v>
       </c>
       <c r="R9" s="4" t="s">
@@ -1694,6 +1719,9 @@
       <c r="T9" s="4" t="s">
         <v>152</v>
       </c>
+      <c r="U9" t="s">
+        <v>198</v>
+      </c>
       <c r="V9" t="s">
         <v>32</v>
       </c>
@@ -1701,15 +1729,15 @@
         <v>0</v>
       </c>
       <c r="X9" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="Y9" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
     </row>
     <row r="10" spans="1:25" ht="96" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B10" t="s">
         <v>39</v>
@@ -1718,25 +1746,25 @@
         <v>41</v>
       </c>
       <c r="D10" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E10">
-        <v>303</v>
+        <v>1234</v>
       </c>
       <c r="F10" s="2">
-        <v>2.4108272399607999E-3</v>
+        <v>9.8183525218207002E-3</v>
       </c>
       <c r="G10">
-        <v>34203</v>
+        <v>34249.5</v>
       </c>
       <c r="H10">
-        <v>7041</v>
+        <v>7298.5</v>
       </c>
       <c r="I10" s="1">
-        <v>0.17790987295142</v>
+        <v>9.4701884701654498E-2</v>
       </c>
       <c r="J10" s="1">
-        <v>1.46487327292562E-2</v>
+        <v>4.5110110659152E-3</v>
       </c>
       <c r="K10" t="b">
         <v>1</v>
@@ -1745,42 +1773,42 @@
         <v>63</v>
       </c>
       <c r="M10" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="N10" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="O10" t="s">
-        <v>95</v>
-      </c>
-      <c r="P10" s="4" t="s">
-        <v>108</v>
+        <v>96</v>
+      </c>
+      <c r="P10" s="5" t="s">
+        <v>109</v>
       </c>
       <c r="R10" s="4" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="S10" s="4" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="T10" s="4" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="V10" t="s">
-        <v>33</v>
+        <v>160</v>
       </c>
       <c r="W10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X10" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="Y10" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
     </row>
     <row r="11" spans="1:25" ht="96" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B11" t="s">
         <v>39</v>
@@ -1789,25 +1817,25 @@
         <v>41</v>
       </c>
       <c r="D11" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E11">
-        <v>1234</v>
+        <v>125</v>
       </c>
       <c r="F11" s="2">
-        <v>9.8183525218207002E-3</v>
+        <v>9.9456569305315001E-4</v>
       </c>
       <c r="G11">
-        <v>34249.5</v>
+        <v>65886</v>
       </c>
       <c r="H11">
-        <v>7298.5</v>
+        <v>9176</v>
       </c>
       <c r="I11" s="1">
-        <v>9.4701884701654498E-2</v>
+        <v>0.11917682861946401</v>
       </c>
       <c r="J11" s="1">
-        <v>4.5110110659152E-3</v>
+        <v>3.6081627011299099E-2</v>
       </c>
       <c r="K11" t="b">
         <v>1</v>
@@ -1816,42 +1844,42 @@
         <v>63</v>
       </c>
       <c r="M11" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="N11" s="3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="O11" t="s">
-        <v>96</v>
-      </c>
-      <c r="P11" s="4" t="s">
-        <v>109</v>
+        <v>97</v>
+      </c>
+      <c r="P11" s="5" t="s">
+        <v>110</v>
       </c>
       <c r="R11" s="4" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="S11" s="4" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="T11" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="V11" t="s">
-        <v>165</v>
+        <v>155</v>
+      </c>
+      <c r="V11" s="3" t="s">
+        <v>161</v>
       </c>
       <c r="W11" t="b">
         <v>1</v>
       </c>
       <c r="X11" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="Y11" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
     </row>
     <row r="12" spans="1:25" ht="96" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B12" t="s">
         <v>39</v>
@@ -1860,25 +1888,25 @@
         <v>41</v>
       </c>
       <c r="D12" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E12">
-        <v>125</v>
+        <v>1363</v>
       </c>
       <c r="F12" s="2">
-        <v>9.9456569305315001E-4</v>
+        <v>1.08447443170516E-2</v>
       </c>
       <c r="G12">
-        <v>65886</v>
+        <v>41165</v>
       </c>
       <c r="H12">
-        <v>9176</v>
+        <v>7923</v>
       </c>
       <c r="I12" s="1">
-        <v>0.11917682861946401</v>
+        <v>0.116135221793027</v>
       </c>
       <c r="J12" s="1">
-        <v>3.6081627011299099E-2</v>
+        <v>3.7882798351347E-3</v>
       </c>
       <c r="K12" t="b">
         <v>1</v>
@@ -1887,42 +1915,42 @@
         <v>63</v>
       </c>
       <c r="M12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="N12" s="3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="O12" t="s">
-        <v>97</v>
-      </c>
-      <c r="P12" s="4" t="s">
-        <v>110</v>
+        <v>98</v>
+      </c>
+      <c r="P12" s="5" t="s">
+        <v>111</v>
       </c>
       <c r="R12" s="4" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="S12" s="4" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="T12" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="V12" s="3" t="s">
-        <v>166</v>
+        <v>156</v>
+      </c>
+      <c r="V12" t="s">
+        <v>162</v>
       </c>
       <c r="W12" t="b">
         <v>1</v>
       </c>
       <c r="X12" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="Y12" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
     </row>
     <row r="13" spans="1:25" ht="96" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B13" t="s">
         <v>39</v>
@@ -1931,25 +1959,25 @@
         <v>41</v>
       </c>
       <c r="D13" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E13">
-        <v>1363</v>
+        <v>303</v>
       </c>
       <c r="F13" s="2">
-        <v>1.08447443170516E-2</v>
+        <v>2.4108272399607999E-3</v>
       </c>
       <c r="G13">
-        <v>41165</v>
+        <v>34203</v>
       </c>
       <c r="H13">
-        <v>7923</v>
+        <v>7041</v>
       </c>
       <c r="I13" s="1">
-        <v>0.116135221793027</v>
+        <v>0.17790987295142</v>
       </c>
       <c r="J13" s="1">
-        <v>3.7882798351347E-3</v>
+        <v>1.46487327292562E-2</v>
       </c>
       <c r="K13" t="b">
         <v>1</v>
@@ -1958,37 +1986,37 @@
         <v>63</v>
       </c>
       <c r="M13" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="N13" s="3" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="O13" t="s">
-        <v>98</v>
-      </c>
-      <c r="P13" s="4" t="s">
-        <v>111</v>
+        <v>95</v>
+      </c>
+      <c r="P13" s="5" t="s">
+        <v>108</v>
       </c>
       <c r="R13" s="4" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="S13" s="4" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="T13" s="4" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="V13" t="s">
-        <v>167</v>
+        <v>33</v>
       </c>
       <c r="W13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X13" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="Y13" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
     </row>
     <row r="14" spans="1:25" ht="112" x14ac:dyDescent="0.2">
@@ -2037,7 +2065,7 @@
       <c r="O14" t="s">
         <v>99</v>
       </c>
-      <c r="P14" s="4" t="s">
+      <c r="P14" s="5" t="s">
         <v>112</v>
       </c>
       <c r="R14" s="4" t="s">
@@ -2050,16 +2078,16 @@
         <v>157</v>
       </c>
       <c r="V14" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="W14" t="b">
         <v>1</v>
       </c>
       <c r="X14" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="Y14" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
     </row>
     <row r="15" spans="1:25" ht="80" x14ac:dyDescent="0.2">
@@ -2108,7 +2136,7 @@
       <c r="O15" t="s">
         <v>100</v>
       </c>
-      <c r="P15" s="4" t="s">
+      <c r="P15" s="5" t="s">
         <v>113</v>
       </c>
       <c r="R15" s="4" t="s">
@@ -2121,20 +2149,24 @@
         <v>158</v>
       </c>
       <c r="V15" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="W15" t="b">
         <v>1</v>
       </c>
       <c r="X15" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="Y15" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Y1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:Y1" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:Y15">
+      <sortCondition ref="N1:N15"/>
+    </sortState>
+  </autoFilter>
   <conditionalFormatting sqref="W1:W1048576">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>TRUE</formula>

</xml_diff>